<commit_message>
Add project configuration files and update report generation
- Created .idea directory with project configuration files including .gitignore, LinearSolvers.iml, misc.xml, modules.xml, and vcs.xml.
- Added REPORT_README.md detailing the LaTeX report structure and compilation instructions.
- Updated results with new comparative images and detailed reports for various methods and matrices.
- Modified summary_table.csv to reflect updated results and performance metrics.
- Adjusted run_tests.py to skip only the gradient method during table and plot generation.
</commit_message>
<xml_diff>
--- a/results/detailed_report_spa1.xlsx
+++ b/results/detailed_report_spa1.xlsx
@@ -473,13 +473,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1.203110531400351e-09</v>
+        <v>1.203110562696275e-09</v>
       </c>
       <c r="E2" t="n">
         <v>200</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1710765000007086</v>
+        <v>0.08433040000090841</v>
       </c>
     </row>
     <row r="3">
@@ -495,13 +495,13 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>2.24808795070259e-08</v>
+        <v>2.248087950909363e-08</v>
       </c>
       <c r="E3" t="n">
         <v>31</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1409016999996311</v>
+        <v>0.09669389999908162</v>
       </c>
     </row>
     <row r="4">
@@ -517,13 +517,13 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>9.82038624805486e-08</v>
+        <v>9.820386166634246e-08</v>
       </c>
       <c r="E4" t="n">
         <v>12919</v>
       </c>
       <c r="F4" t="n">
-        <v>7.647178300000633</v>
+        <v>3.622965099999419</v>
       </c>
     </row>
     <row r="5">
@@ -539,13 +539,13 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1.852435597686972e-09</v>
+        <v>1.852435171110543e-09</v>
       </c>
       <c r="E5" t="n">
         <v>313</v>
       </c>
       <c r="F5" t="n">
-        <v>2.438313700000435</v>
+        <v>1.758664600001794</v>
       </c>
     </row>
     <row r="6">
@@ -561,13 +561,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1.319840444579099e-07</v>
+        <v>1.319840447022883e-07</v>
       </c>
       <c r="E6" t="n">
         <v>177</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1445136000002094</v>
+        <v>0.05593130000124802</v>
       </c>
     </row>
     <row r="7">
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1.709732900381708e-06</v>
+        <v>1.709732900390593e-06</v>
       </c>
       <c r="E7" t="n">
         <v>24</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1128467999997156</v>
+        <v>0.05153760000030161</v>
       </c>
     </row>
     <row r="8">
@@ -605,13 +605,13 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>9.816363743993126e-06</v>
+        <v>9.81636374318044e-06</v>
       </c>
       <c r="E8" t="n">
         <v>8233</v>
       </c>
       <c r="F8" t="n">
-        <v>4.769082400000116</v>
+        <v>1.870501299999887</v>
       </c>
     </row>
     <row r="9">
@@ -627,13 +627,13 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>1.824978864492149e-07</v>
+        <v>1.82497886508391e-07</v>
       </c>
       <c r="E9" t="n">
         <v>247</v>
       </c>
       <c r="F9" t="n">
-        <v>2.216449600000487</v>
+        <v>1.165423099999316</v>
       </c>
     </row>
     <row r="10">
@@ -649,13 +649,13 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>2.552909277601956e-05</v>
+        <v>2.552909277634323e-05</v>
       </c>
       <c r="E10" t="n">
         <v>134</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1079528000000209</v>
+        <v>0.03071329999875161</v>
       </c>
     </row>
     <row r="11">
@@ -671,13 +671,13 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.000129969395859719</v>
+        <v>0.0001299693958597223</v>
       </c>
       <c r="E11" t="n">
         <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>0.07097370000064984</v>
+        <v>0.03681219999998575</v>
       </c>
     </row>
     <row r="12">
@@ -693,13 +693,13 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0009680457310610326</v>
+        <v>0.0009680457310602736</v>
       </c>
       <c r="E12" t="n">
         <v>3577</v>
       </c>
       <c r="F12" t="n">
-        <v>1.765021299999717</v>
+        <v>0.7821442999993451</v>
       </c>
     </row>
     <row r="13">
@@ -715,13 +715,13 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1.79792954354708e-05</v>
+        <v>1.79792954346363e-05</v>
       </c>
       <c r="E13" t="n">
         <v>181</v>
       </c>
       <c r="F13" t="n">
-        <v>1.366011799999796</v>
+        <v>0.8775707999993756</v>
       </c>
     </row>
     <row r="14">
@@ -737,13 +737,13 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02078976000995673</v>
+        <v>0.02078976000995638</v>
       </c>
       <c r="E14" t="n">
         <v>49</v>
       </c>
       <c r="F14" t="n">
-        <v>0.02363409999998112</v>
+        <v>0.01128959999914514</v>
       </c>
     </row>
     <row r="15">
@@ -765,7 +765,7 @@
         <v>9</v>
       </c>
       <c r="F15" t="n">
-        <v>0.03791689999980008</v>
+        <v>0.01928319999933592</v>
       </c>
     </row>
     <row r="16">
@@ -781,13 +781,13 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0.03457470077301093</v>
+        <v>0.03457470077301085</v>
       </c>
       <c r="E16" t="n">
         <v>143</v>
       </c>
       <c r="F16" t="n">
-        <v>0.09380669999973179</v>
+        <v>0.03217589999985648</v>
       </c>
     </row>
     <row r="17">
@@ -803,13 +803,13 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.001771281148305467</v>
+        <v>0.001771281148305705</v>
       </c>
       <c r="E17" t="n">
         <v>115</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8983594000001176</v>
+        <v>0.5265241999986756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>